<commit_message>
fixed backtest start date to 2024
</commit_message>
<xml_diff>
--- a/exports/gilt/gilt_curveTradesRecap_avgTrades.xlsx
+++ b/exports/gilt/gilt_curveTradesRecap_avgTrades.xlsx
@@ -505,13 +505,13 @@
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4">
-        <v>13.9</v>
+        <v>7.8</v>
       </c>
       <c r="E3" s="4">
-        <v>14.3</v>
+        <v>7</v>
       </c>
       <c r="F3" s="5">
-        <v>17</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="15.5" customHeight="1">
@@ -520,13 +520,13 @@
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4">
-        <v>16.8</v>
+        <v>8.4</v>
       </c>
       <c r="E4" s="4">
-        <v>18.9</v>
+        <v>8.6</v>
       </c>
       <c r="F4" s="5">
-        <v>18.2</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="15.5" customHeight="1">
@@ -536,10 +536,10 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4">
-        <v>18.4</v>
+        <v>11.5</v>
       </c>
       <c r="F5" s="5">
-        <v>16.9</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="15.5" customHeight="1">
@@ -550,7 +550,7 @@
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="5">
-        <v>14.5</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="5" customHeight="1"/>

</xml_diff>